<commit_message>
Fixed import cards not passing path chages to config services.
</commit_message>
<xml_diff>
--- a/EinsatzPlanung/Assets/Excel/Ferien.xlsx
+++ b/EinsatzPlanung/Assets/Excel/Ferien.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex\source\repos\EinsatzPlanung\EinsatzPlanung\Assets\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3FFB802-8409-4620-AACA-7DEF94BDAEFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD39DB10-1330-4063-9356-946BC7362FE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11565" yWindow="555" windowWidth="15180" windowHeight="15645" xr2:uid="{93971DC9-9131-4D11-831F-804A5976373C}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{93971DC9-9131-4D11-831F-804A5976373C}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -460,6 +460,9 @@
       <c r="A3" s="3">
         <v>45753</v>
       </c>
+      <c r="B3" s="3">
+        <v>45753</v>
+      </c>
       <c r="C3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="1"/>

</xml_diff>